<commit_message>
mtf code is done, crazy one
</commit_message>
<xml_diff>
--- a/Electromagnetismo/practica4carretes/p4electro.xlsx
+++ b/Electromagnetismo/practica4carretes/p4electro.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="33">
   <si>
     <t>N</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t>B teorico</t>
+  </si>
+  <si>
+    <t>inc'</t>
   </si>
   <si>
     <t>I(A)</t>
@@ -116,9 +119,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="d.m"/>
-  </numFmts>
   <fonts count="2">
     <font>
       <sz val="10.0"/>
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -190,10 +190,6 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="4" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -302,11 +298,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1959601235"/>
-        <c:axId val="476344087"/>
+        <c:axId val="1720112591"/>
+        <c:axId val="1494245639"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1959601235"/>
+        <c:axId val="1720112591"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -381,10 +377,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="476344087"/>
+        <c:crossAx val="1494245639"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="476344087"/>
+        <c:axId val="1494245639"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -459,7 +455,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1959601235"/>
+        <c:crossAx val="1720112591"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -568,11 +564,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1460412182"/>
-        <c:axId val="1242467718"/>
+        <c:axId val="1853140790"/>
+        <c:axId val="1321138146"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1460412182"/>
+        <c:axId val="1853140790"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -647,10 +643,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1242467718"/>
+        <c:crossAx val="1321138146"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1242467718"/>
+        <c:axId val="1321138146"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -725,7 +721,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1460412182"/>
+        <c:crossAx val="1853140790"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -1768,6 +1764,137 @@
         <v>0</v>
       </c>
     </row>
+    <row r="29">
+      <c r="D29" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="D30" s="2">
+        <f t="shared" ref="D30:D50" si="6">(0.02*C6)+0.01</f>
+        <v>0.0376</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="D31" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0336</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="D32" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0322</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="D33" s="2">
+        <f t="shared" si="6"/>
+        <v>0.029</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="D34" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0258</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="D35" s="2">
+        <f t="shared" si="6"/>
+        <v>0.023</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="D36" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0194</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="D37" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0156</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="D38" s="2">
+        <f t="shared" si="6"/>
+        <v>0.014</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="D39" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0126</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="D40" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0238</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="D41" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0394</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="D42" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0416</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="D43" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0426</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="D44" s="2">
+        <f t="shared" si="6"/>
+        <v>0.044</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="D45" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0442</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="D46" s="2">
+        <f t="shared" si="6"/>
+        <v>0.021</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="D47" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0178</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="D48" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0268</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="D49" s="2">
+        <f t="shared" si="6"/>
+        <v>0.0306</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="D50" s="2">
+        <f t="shared" si="6"/>
+        <v>0.036</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -1782,16 +1909,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2">
@@ -1799,8 +1926,8 @@
         <v>1.38</v>
       </c>
       <c r="B2" s="2">
-        <f t="shared" ref="B2:B22" si="1">A2*(2.5/100)+0.1</f>
-        <v>0.1345</v>
+        <f t="shared" ref="B2:B22" si="1">(0.02*A2)+0.01</f>
+        <v>0.0376</v>
       </c>
       <c r="C2" s="1">
         <v>-2.28</v>
@@ -1816,7 +1943,7 @@
       </c>
       <c r="B3" s="2">
         <f t="shared" si="1"/>
-        <v>0.1295</v>
+        <v>0.0336</v>
       </c>
       <c r="C3" s="1">
         <v>-1.97</v>
@@ -1832,7 +1959,7 @@
       </c>
       <c r="B4" s="2">
         <f t="shared" si="1"/>
-        <v>0.12775</v>
+        <v>0.0322</v>
       </c>
       <c r="C4" s="1">
         <v>-1.84</v>
@@ -1848,7 +1975,7 @@
       </c>
       <c r="B5" s="2">
         <f t="shared" si="1"/>
-        <v>0.12375</v>
+        <v>0.029</v>
       </c>
       <c r="C5" s="1">
         <v>-1.6</v>
@@ -1864,7 +1991,7 @@
       </c>
       <c r="B6" s="2">
         <f t="shared" si="1"/>
-        <v>0.11975</v>
+        <v>0.0258</v>
       </c>
       <c r="C6" s="1">
         <v>-1.33</v>
@@ -1880,7 +2007,7 @@
       </c>
       <c r="B7" s="2">
         <f t="shared" si="1"/>
-        <v>0.11625</v>
+        <v>0.023</v>
       </c>
       <c r="C7" s="1">
         <v>-1.11</v>
@@ -1896,7 +2023,7 @@
       </c>
       <c r="B8" s="2">
         <f t="shared" si="1"/>
-        <v>0.11175</v>
+        <v>0.0194</v>
       </c>
       <c r="C8" s="1">
         <v>-0.79</v>
@@ -1912,7 +2039,7 @@
       </c>
       <c r="B9" s="2">
         <f t="shared" si="1"/>
-        <v>0.107</v>
+        <v>0.0156</v>
       </c>
       <c r="C9" s="1">
         <v>-0.53</v>
@@ -1928,7 +2055,7 @@
       </c>
       <c r="B10" s="2">
         <f t="shared" si="1"/>
-        <v>0.105</v>
+        <v>0.014</v>
       </c>
       <c r="C10" s="1">
         <v>-0.36</v>
@@ -1944,7 +2071,7 @@
       </c>
       <c r="B11" s="2">
         <f t="shared" si="1"/>
-        <v>0.10325</v>
+        <v>0.0126</v>
       </c>
       <c r="C11" s="1">
         <v>-0.24</v>
@@ -1960,7 +2087,7 @@
       </c>
       <c r="B12" s="2">
         <f t="shared" si="1"/>
-        <v>0.11725</v>
+        <v>0.0238</v>
       </c>
       <c r="C12" s="1">
         <v>-1.18</v>
@@ -1976,7 +2103,7 @@
       </c>
       <c r="B13" s="2">
         <f t="shared" si="1"/>
-        <v>0.13675</v>
+        <v>0.0394</v>
       </c>
       <c r="C13" s="1">
         <v>-2.42</v>
@@ -1992,7 +2119,7 @@
       </c>
       <c r="B14" s="2">
         <f t="shared" si="1"/>
-        <v>0.1395</v>
+        <v>0.0416</v>
       </c>
       <c r="C14" s="1">
         <v>-2.61</v>
@@ -2008,7 +2135,7 @@
       </c>
       <c r="B15" s="2">
         <f t="shared" si="1"/>
-        <v>0.14075</v>
+        <v>0.0426</v>
       </c>
       <c r="C15" s="1">
         <v>-2.7</v>
@@ -2024,7 +2151,7 @@
       </c>
       <c r="B16" s="2">
         <f t="shared" si="1"/>
-        <v>0.1425</v>
+        <v>0.044</v>
       </c>
       <c r="C16" s="1">
         <v>-2.8</v>
@@ -2040,7 +2167,7 @@
       </c>
       <c r="B17" s="2">
         <f t="shared" si="1"/>
-        <v>0.14275</v>
+        <v>0.0442</v>
       </c>
       <c r="C17" s="1">
         <v>-2.83</v>
@@ -2056,7 +2183,7 @@
       </c>
       <c r="B18" s="2">
         <f t="shared" si="1"/>
-        <v>0.11375</v>
+        <v>0.021</v>
       </c>
       <c r="C18" s="1">
         <v>-0.94</v>
@@ -2072,7 +2199,7 @@
       </c>
       <c r="B19" s="2">
         <f t="shared" si="1"/>
-        <v>0.10975</v>
+        <v>0.0178</v>
       </c>
       <c r="C19" s="1">
         <v>-0.67</v>
@@ -2088,7 +2215,7 @@
       </c>
       <c r="B20" s="2">
         <f t="shared" si="1"/>
-        <v>0.121</v>
+        <v>0.0268</v>
       </c>
       <c r="C20" s="1">
         <v>-1.45</v>
@@ -2104,7 +2231,7 @@
       </c>
       <c r="B21" s="2">
         <f t="shared" si="1"/>
-        <v>0.12575</v>
+        <v>0.0306</v>
       </c>
       <c r="C21" s="1">
         <v>-1.74</v>
@@ -2120,7 +2247,7 @@
       </c>
       <c r="B22" s="2">
         <f t="shared" si="1"/>
-        <v>0.1325</v>
+        <v>0.036</v>
       </c>
       <c r="C22" s="1">
         <v>-2.16</v>
@@ -2151,7 +2278,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2160,16 +2287,16 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2">
@@ -2205,16 +2332,16 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>9</v>
@@ -2223,13 +2350,13 @@
         <v>10</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -2718,16 +2845,16 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>9</v>
@@ -2736,13 +2863,13 @@
         <v>10</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>12</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24">
@@ -3261,16 +3388,16 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>9</v>
@@ -3279,13 +3406,13 @@
         <v>10</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>12</v>
       </c>
       <c r="I42" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43">
@@ -3299,8 +3426,8 @@
         <v>322.0</v>
       </c>
       <c r="D43" s="8">
-        <f t="shared" ref="D43:D57" si="7">-$A$6+C43</f>
-        <v>28</v>
+        <f t="shared" ref="D43:D57" si="7">-$A$43+C43</f>
+        <v>0</v>
       </c>
       <c r="E43" s="7">
         <v>1.5</v>
@@ -3330,7 +3457,7 @@
       </c>
       <c r="D44" s="8">
         <f t="shared" si="7"/>
-        <v>36</v>
+        <v>8</v>
       </c>
       <c r="E44" s="7">
         <v>1.5</v>
@@ -3360,7 +3487,7 @@
       </c>
       <c r="D45" s="8">
         <f t="shared" si="7"/>
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="E45" s="7">
         <v>1.5</v>
@@ -3390,7 +3517,7 @@
       </c>
       <c r="D46" s="8">
         <f t="shared" si="7"/>
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="E46" s="7">
         <v>1.5</v>
@@ -3420,7 +3547,7 @@
       </c>
       <c r="D47" s="8">
         <f t="shared" si="7"/>
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="E47" s="7">
         <v>1.5</v>
@@ -3450,7 +3577,7 @@
       </c>
       <c r="D48" s="8">
         <f t="shared" si="7"/>
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="E48" s="7">
         <v>1.5</v>
@@ -3480,7 +3607,7 @@
       </c>
       <c r="D49" s="8">
         <f t="shared" si="7"/>
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E49" s="7">
         <v>1.5</v>
@@ -3510,7 +3637,7 @@
       </c>
       <c r="D50" s="8">
         <f t="shared" si="7"/>
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E50" s="7">
         <v>1.5</v>
@@ -3540,7 +3667,7 @@
       </c>
       <c r="D51" s="8">
         <f t="shared" si="7"/>
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="E51" s="7">
         <v>1.5</v>
@@ -3570,7 +3697,7 @@
       </c>
       <c r="D52" s="8">
         <f t="shared" si="7"/>
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="E52" s="7">
         <v>1.5</v>
@@ -3600,14 +3727,14 @@
       </c>
       <c r="D53" s="8">
         <f t="shared" si="7"/>
-        <v>126</v>
-      </c>
-      <c r="E53" s="9">
-        <v>46143.0</v>
-      </c>
-      <c r="F53" s="10">
+        <v>98</v>
+      </c>
+      <c r="E53" s="7">
+        <v>1.5</v>
+      </c>
+      <c r="F53" s="8">
         <f t="shared" si="8"/>
-        <v>1153.675</v>
+        <v>0.1375</v>
       </c>
       <c r="G53" s="7">
         <v>-1.84</v>
@@ -3630,7 +3757,7 @@
       </c>
       <c r="D54" s="8">
         <f t="shared" si="7"/>
-        <v>136</v>
+        <v>108</v>
       </c>
       <c r="E54" s="7">
         <v>1.5</v>
@@ -3660,7 +3787,7 @@
       </c>
       <c r="D55" s="8">
         <f t="shared" si="7"/>
-        <v>146</v>
+        <v>118</v>
       </c>
       <c r="E55" s="7">
         <v>1.5</v>
@@ -3690,7 +3817,7 @@
       </c>
       <c r="D56" s="8">
         <f t="shared" si="7"/>
-        <v>156</v>
+        <v>128</v>
       </c>
       <c r="E56" s="7">
         <v>1.5</v>
@@ -3720,7 +3847,7 @@
       </c>
       <c r="D57" s="8">
         <f t="shared" si="7"/>
-        <v>166</v>
+        <v>138</v>
       </c>
       <c r="E57" s="7">
         <v>1.5</v>
@@ -3752,16 +3879,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>9</v>
@@ -3770,19 +3897,19 @@
         <v>10</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="I1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2">
@@ -4394,49 +4521,49 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11">
+      <c r="A18" s="9">
         <v>296.0</v>
       </c>
-      <c r="B18" s="11">
-        <v>10.5</v>
-      </c>
-      <c r="C18" s="11">
+      <c r="B18" s="9">
+        <v>10.5</v>
+      </c>
+      <c r="C18" s="9">
         <v>290.0</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="10">
         <f t="shared" si="1"/>
         <v>-6</v>
       </c>
-      <c r="E18" s="11">
-        <v>1.5</v>
-      </c>
-      <c r="F18" s="12">
-        <f t="shared" si="2"/>
-        <v>0.1375</v>
-      </c>
-      <c r="G18" s="11">
+      <c r="E18" s="9">
+        <v>1.5</v>
+      </c>
+      <c r="F18" s="10">
+        <f t="shared" si="2"/>
+        <v>0.1375</v>
+      </c>
+      <c r="G18" s="9">
         <v>-0.15</v>
       </c>
-      <c r="H18" s="12">
-        <f t="shared" si="3"/>
-        <v>0.002886751346</v>
-      </c>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="M18" s="12"/>
-      <c r="N18" s="12"/>
-      <c r="O18" s="12"/>
-      <c r="P18" s="12"/>
-      <c r="Q18" s="12"/>
-      <c r="R18" s="12"/>
-      <c r="S18" s="12"/>
-      <c r="T18" s="12"/>
-      <c r="U18" s="12"/>
-      <c r="V18" s="12"/>
-      <c r="W18" s="12"/>
-      <c r="X18" s="12"/>
-      <c r="Y18" s="12"/>
-      <c r="Z18" s="12"/>
+      <c r="H18" s="10">
+        <f t="shared" si="3"/>
+        <v>0.002886751346</v>
+      </c>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="M18" s="10"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="10"/>
+      <c r="S18" s="10"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="10"/>
+      <c r="V18" s="10"/>
+      <c r="W18" s="10"/>
+      <c r="X18" s="10"/>
+      <c r="Y18" s="10"/>
+      <c r="Z18" s="10"/>
     </row>
     <row r="19">
       <c r="A19" s="3">

</xml_diff>